<commit_message>
Alteração conforme deliberação XXX - 30/03/2022
Teste
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\Documents\1.CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-vale\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m7522667\Documents\code\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
   <si>
     <t>projeto</t>
   </si>
@@ -217,9 +217,6 @@
   </si>
   <si>
     <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
-  </si>
-  <si>
-    <t>Implantação de Fábrica de Software para construção de sistema de governança ambiental</t>
   </si>
   <si>
     <t>Ressarcimentos e contratações temporárias</t>
@@ -602,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -1221,7 +1218,7 @@
         <v>49</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D44" s="1">
         <v>100000000</v>
@@ -1263,7 +1260,7 @@
         <v>52</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D47" s="1">
         <v>210000000</v>
@@ -1365,20 +1362,6 @@
       </c>
       <c r="D54" s="1">
         <v>749679</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>9288213</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D55" s="1">
-        <v>23000005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Teste validação do repositório
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
+  </si>
+  <si>
+    <t>z.Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
@@ -1166,7 +1169,7 @@
         <v>49</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="D43" s="1">
         <v>100000000</v>

</xml_diff>

<commit_message>
testa validação linhas 41 e 43
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\Documents\1.CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="63">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -212,7 +212,10 @@
     <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
   </si>
   <si>
-    <t>z.Ressarcimentos e contratações temporárias</t>
+    <t>II</t>
+  </si>
+  <si>
+    <t>Z.Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1144,7 @@
         <v>51</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="D41" s="1">
         <v>99720000</v>
@@ -1169,7 +1172,7 @@
         <v>49</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D43" s="1">
         <v>100000000</v>

</xml_diff>

<commit_message>
corrige erro linha 43
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\Documents\1.CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -212,10 +212,7 @@
     <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
   </si>
   <si>
-    <t>II</t>
-  </si>
-  <si>
-    <t>Z.Ressarcimentos e contratações temporárias</t>
+    <t>Estruturas de Apoio</t>
   </si>
 </sst>
 </file>
@@ -1172,7 +1169,7 @@
         <v>49</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="D43" s="1">
         <v>100000000</v>

</xml_diff>

<commit_message>
corrige erro linha 41
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -210,9 +210,6 @@
   </si>
   <si>
     <t>Fortalecimento da estrutura de fiscalização do Sistema Estadual de Meio Ambiente</t>
-  </si>
-  <si>
-    <t>Estruturas de Apoio</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1138,7 @@
         <v>51</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="D41" s="1">
         <v>99720000</v>
@@ -1334,6 +1331,6 @@
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.51180555555555496" right="0.51180555555555496" top="0.78749999999999998" bottom="0.78749999999999998" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" firstPageNumber="0" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Acrescenta linha para teste
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="61">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -561,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -1340,6 +1340,20 @@
         <v>800000</v>
       </c>
     </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56" s="3">
+        <v>9288214</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D56" s="1">
+        <v>800000</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="A2:D56">
     <sortCondition ref="A1"/>

</xml_diff>

<commit_message>
Alteração conforme deliberação xx/2022
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C9BE0A-73EF-4AEB-AEBB-9D999849DAA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744E0528-A62A-4563-9119-6D9C7DDE2703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -591,7 +591,7 @@
   <sheetFormatPr defaultColWidth="28.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
-    <col min="2" max="2" width="83.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="90.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="23.85546875" customWidth="1"/>
     <col min="4" max="4" width="28.7109375" style="2"/>
   </cols>
@@ -1349,7 +1349,7 @@
         <v>5</v>
       </c>
       <c r="D54" s="2">
-        <v>810000</v>
+        <v>9000000</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Alteração conforme deliberação 06 de 28/04/2022
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744E0528-A62A-4563-9119-6D9C7DDE2703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AAAEBD5-7333-4A9E-B73D-703146301E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1349,7 +1349,7 @@
         <v>5</v>
       </c>
       <c r="D54" s="2">
-        <v>9000000</v>
+        <v>8000000</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Corrige linha 42 - Coluna Anexo
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\Teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DE48F30-5383-4F35-A985-9D528850439A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3C2E90-E5A2-47AF-A464-441E874BEA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="61">
   <si>
     <t>codigo_projeto</t>
   </si>
@@ -211,9 +211,6 @@
   </si>
   <si>
     <t>Plano de Desenvolvimento da Cadeia Agropecuária</t>
-  </si>
-  <si>
-    <t>z.Ressarcimentos e contratações temporárias</t>
   </si>
 </sst>
 </file>
@@ -1181,7 +1178,7 @@
         <v>46</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="D42" s="2">
         <v>210000000</v>

</xml_diff>

<commit_message>
Limites Projetos - Deliberação nº 06
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -262,7 +262,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -271,6 +271,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,723 +578,723 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>9288212</v>
+      <c r="A2" s="4">
+        <v>9288130</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" s="3">
-        <v>2050000000</v>
+        <v>450000000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="4">
         <v>9288130</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C3" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="3">
-        <v>450000000</v>
+        <v>300000000</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="e">
-        <v>#N/A</v>
+      <c r="A4" s="4">
+        <v>9288132</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="3">
-        <v>427970000</v>
+        <v>700000000</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>9288132</v>
+      <c r="A5" s="4">
+        <v>9288133</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D5" s="3">
-        <v>300000000</v>
+        <v>98860000</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>9288180</v>
+      <c r="A6" s="4">
+        <v>9288134</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3">
-        <v>3072030000</v>
+        <v>1345000</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>9288133</v>
+      <c r="A7" s="4">
+        <v>9288135</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D7" s="3">
-        <v>700000000</v>
+        <v>111480000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>9288185</v>
+      <c r="A8" s="4">
+        <v>9288136</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="3">
-        <v>2000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <v>9288176</v>
+      <c r="A9" s="4">
+        <v>9288137</v>
       </c>
       <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3">
+        <v>39614000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4">
+        <v>9288138</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3">
+        <v>3200000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4">
+        <v>9288139</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>9288141</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3">
+        <v>29712000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>9288142</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="3">
+        <v>728000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>9288143</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="3">
+        <v>49000000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>9288144</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="3">
+        <v>45345000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>9288145</v>
+      </c>
+      <c r="B16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="3">
+        <v>14817323</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>9288147</v>
+      </c>
+      <c r="B17" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="3">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>9288148</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="3">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="4">
+        <v>9288149</v>
+      </c>
+      <c r="B19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="3">
+        <v>10671300</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>9288150</v>
+      </c>
+      <c r="B20" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="3">
+        <v>15130000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>9288152</v>
+      </c>
+      <c r="B21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="3">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="4">
+        <v>9288153</v>
+      </c>
+      <c r="B22" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" s="3">
+        <v>650000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="4">
+        <v>9288154</v>
+      </c>
+      <c r="B23" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="3">
+        <v>5100000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>9288155</v>
+      </c>
+      <c r="B24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3773400</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>9288167</v>
+      </c>
+      <c r="B25" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="3">
+        <v>130000000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="4">
+        <v>9288168</v>
+      </c>
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="3">
+        <v>43368482</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="4">
+        <v>9288169</v>
+      </c>
+      <c r="B27" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="3">
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="3">
         <f>8700000+14431467.96</f>
         <v>23131467.960000001</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9288139</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="3">
-        <v>3200000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>9288135</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D11" s="3">
-        <v>1345000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>9288169</v>
-      </c>
-      <c r="B12" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="3">
-        <v>43368482</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>9288168</v>
-      </c>
-      <c r="B13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="3">
-        <v>130000000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>9288167</v>
-      </c>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="3">
-        <v>3773400</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
-        <v>9288155</v>
-      </c>
-      <c r="B15" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" t="s">
-        <v>8</v>
-      </c>
-      <c r="D15" s="3">
-        <v>5100000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16">
-        <v>9288136</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" t="s">
-        <v>8</v>
-      </c>
-      <c r="D16" s="3">
-        <v>111480000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>9288214</v>
-      </c>
-      <c r="B17" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" t="s">
-        <v>8</v>
-      </c>
-      <c r="D17" s="3">
-        <v>199489167.000002</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>9288209</v>
-      </c>
-      <c r="B18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" t="s">
-        <v>8</v>
-      </c>
-      <c r="D18" s="3">
-        <v>1200000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19">
-        <v>9288147</v>
-      </c>
-      <c r="B19" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="3">
-        <v>14817323</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>9288141</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" t="s">
-        <v>8</v>
-      </c>
-      <c r="D20" s="3">
-        <v>500000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21">
-        <v>9288142</v>
-      </c>
-      <c r="B21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="3">
-        <v>29712000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22">
-        <v>9288193</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" t="s">
-        <v>8</v>
-      </c>
-      <c r="D22" s="3">
-        <v>3900000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>9288194</v>
-      </c>
-      <c r="B23" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" t="s">
-        <v>8</v>
-      </c>
-      <c r="D23" s="3">
-        <v>3600000</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24">
-        <v>9288149</v>
-      </c>
-      <c r="B24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="3">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25">
-        <v>9288143</v>
-      </c>
-      <c r="B25" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="3">
-        <v>728000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>9288144</v>
-      </c>
-      <c r="B26" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D26" s="3">
-        <v>49000000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27">
-        <v>9288196</v>
-      </c>
-      <c r="B27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" t="s">
-        <v>8</v>
-      </c>
-      <c r="D27" s="3">
-        <v>42412000</v>
-      </c>
-    </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28">
-        <v>9288145</v>
+      <c r="A28" s="4">
+        <v>9288176</v>
       </c>
       <c r="B28" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
         <v>8</v>
       </c>
       <c r="D28" s="3">
-        <v>45345000</v>
+        <v>100370000</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>9288137</v>
+      <c r="A29" s="4">
+        <v>9288177</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
       </c>
       <c r="D29" s="3">
-        <v>100000000</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>9288148</v>
-      </c>
-      <c r="B30" t="s">
-        <v>31</v>
-      </c>
-      <c r="C30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="3">
-        <v>3000000</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>9288138</v>
-      </c>
-      <c r="B31" t="s">
-        <v>32</v>
-      </c>
-      <c r="C31" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="3">
-        <v>39614000</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>9288150</v>
-      </c>
-      <c r="B32" t="s">
-        <v>33</v>
-      </c>
-      <c r="C32" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="3">
-        <v>10671300</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>9321270</v>
-      </c>
-      <c r="B33" t="s">
-        <v>34</v>
-      </c>
-      <c r="C33" t="s">
-        <v>8</v>
-      </c>
-      <c r="D33" s="3">
-        <v>800000</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>9288152</v>
-      </c>
-      <c r="B34" t="s">
-        <v>35</v>
-      </c>
-      <c r="C34" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="3">
-        <v>15130000</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>9288153</v>
-      </c>
-      <c r="B35" t="s">
-        <v>36</v>
-      </c>
-      <c r="C35" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="3">
-        <v>3000000</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>9288154</v>
-      </c>
-      <c r="B36" t="s">
-        <v>37</v>
-      </c>
-      <c r="C36" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="3">
-        <v>650000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <v>9288210</v>
-      </c>
-      <c r="B37" t="s">
-        <v>38</v>
-      </c>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-      <c r="D37" s="3">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <v>9288211</v>
-      </c>
-      <c r="B38" t="s">
-        <v>39</v>
-      </c>
-      <c r="C38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="3">
-        <v>3200000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <v>9288177</v>
-      </c>
-      <c r="B39" t="s">
-        <v>57</v>
-      </c>
-      <c r="C39" t="s">
-        <v>8</v>
-      </c>
-      <c r="D39" s="3">
-        <v>100370000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <v>9288177</v>
-      </c>
-      <c r="B40" t="s">
-        <v>56</v>
-      </c>
-      <c r="C40" t="s">
-        <v>8</v>
-      </c>
-      <c r="D40" s="3">
         <f>1048250000+59300000</f>
         <v>1107550000</v>
       </c>
     </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="4">
+        <v>9288178</v>
+      </c>
+      <c r="B30" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="3">
+        <v>253000000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="4">
+        <v>9288179</v>
+      </c>
+      <c r="B31" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="3">
+        <v>45000000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="4">
+        <v>9288180</v>
+      </c>
+      <c r="B32" t="s">
+        <v>6</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="3">
+        <v>3072030000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="4">
+        <v>9288181</v>
+      </c>
+      <c r="B33" t="s">
+        <v>43</v>
+      </c>
+      <c r="C33" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="3">
+        <v>75352000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="4">
+        <v>9288182</v>
+      </c>
+      <c r="B34" t="s">
+        <v>44</v>
+      </c>
+      <c r="C34" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="3">
+        <v>7000000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="4">
+        <v>9288183</v>
+      </c>
+      <c r="B35" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="3">
+        <v>8000000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="4">
+        <v>9288185</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="3">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="4">
+        <v>9288186</v>
+      </c>
+      <c r="B37" t="s">
+        <v>47</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37" s="3">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="4">
+        <v>9288187</v>
+      </c>
+      <c r="B38" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="3">
+        <v>36000000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="4">
+        <v>9288188</v>
+      </c>
+      <c r="B39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="3">
+        <v>8647600</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="4">
+        <v>9288189</v>
+      </c>
+      <c r="B40" t="s">
+        <v>50</v>
+      </c>
+      <c r="C40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="3">
+        <v>300000</v>
+      </c>
+    </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <v>9288178</v>
+      <c r="A41" s="4">
+        <v>9288190</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C41" t="s">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="D41" s="3">
-        <v>253000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <v>9288179</v>
+      <c r="A42" s="4">
+        <v>9288191</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="D42" s="3">
-        <v>45000000</v>
+        <v>210000000</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <v>9288134</v>
+      <c r="A43" s="4">
+        <v>9288192</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C43" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="D43" s="3">
-        <v>98860000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <v>9288181</v>
+      <c r="A44" s="4">
+        <v>9288193</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="C44" t="s">
         <v>8</v>
       </c>
       <c r="D44" s="3">
-        <v>75352000</v>
+        <v>3900000</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <v>9288183</v>
+      <c r="A45" s="4">
+        <v>9288194</v>
       </c>
       <c r="B45" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="C45" t="s">
         <v>8</v>
       </c>
       <c r="D45" s="3">
-        <v>8000000</v>
+        <v>3600000</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <v>9288182</v>
+      <c r="A46" s="4">
+        <v>9288195</v>
       </c>
       <c r="B46" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C46" t="s">
         <v>8</v>
       </c>
       <c r="D46" s="3">
-        <v>7000000</v>
+        <v>749679</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47">
+      <c r="A47" s="4">
+        <v>9288196</v>
+      </c>
+      <c r="B47" t="s">
+        <v>27</v>
+      </c>
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="3">
+        <v>42412000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48" s="4">
         <v>9288198</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>46</v>
       </c>
-      <c r="C47" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" s="3">
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="3">
         <v>985935044</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <v>9288186</v>
-      </c>
-      <c r="B48" t="s">
-        <v>47</v>
-      </c>
-      <c r="C48" t="s">
-        <v>8</v>
-      </c>
-      <c r="D48" s="3">
-        <v>3000000</v>
-      </c>
-    </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <v>9288187</v>
+      <c r="A49" s="4">
+        <v>9288209</v>
       </c>
       <c r="B49" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="C49" t="s">
         <v>8</v>
       </c>
       <c r="D49" s="3">
-        <v>36000000</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50">
-        <v>9288188</v>
+      <c r="A50" s="4">
+        <v>9288210</v>
       </c>
       <c r="B50" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="C50" t="s">
         <v>8</v>
       </c>
       <c r="D50" s="3">
-        <v>8647600</v>
+        <v>2500000</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51">
-        <v>9288189</v>
+      <c r="A51" s="4">
+        <v>9288211</v>
       </c>
       <c r="B51" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C51" t="s">
         <v>8</v>
       </c>
       <c r="D51" s="3">
-        <v>300000</v>
+        <v>3200000</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52">
-        <v>9288195</v>
+      <c r="A52" s="4">
+        <v>9288212</v>
       </c>
       <c r="B52" t="s">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="C52" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D52" s="3">
-        <v>749679</v>
+        <v>2050000000</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53">
+      <c r="A53" s="4">
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
@@ -1305,45 +1308,45 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54">
-        <v>9288190</v>
+      <c r="A54" s="4">
+        <v>9288214</v>
       </c>
       <c r="B54" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
       <c r="C54" t="s">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="D54" s="3">
-        <v>100000000</v>
+        <v>199489167.000002</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55">
-        <v>9288192</v>
+      <c r="A55" s="4">
+        <v>9321270</v>
       </c>
       <c r="B55" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="C55" t="s">
-        <v>59</v>
+        <v>8</v>
       </c>
       <c r="D55" s="3">
-        <v>100000000</v>
+        <v>800000</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>9288191</v>
+      <c r="A56" t="e">
+        <v>#N/A</v>
       </c>
       <c r="B56" t="s">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="C56" t="s">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="D56" s="3">
-        <v>210000000</v>
+        <v>427970000</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -1361,6 +1364,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState ref="A2:D57">
+    <sortCondition ref="A1"/>
+  </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajusta dados dos valores
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -1,23 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugos\Desktop\Documentos Brumadinho\projeto VALE CGE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21EED634-49F9-4F5F-AA34-3A8CAA58D760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="6750" tabRatio="867"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="projetos" sheetId="9" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -221,7 +232,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
@@ -262,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -271,9 +282,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -554,7 +562,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -578,7 +586,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
+      <c r="A2">
         <v>9288130</v>
       </c>
       <c r="B2" t="s">
@@ -592,7 +600,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
+      <c r="A3">
         <v>9288130</v>
       </c>
       <c r="B3" t="s">
@@ -606,7 +614,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+      <c r="A4">
         <v>9288132</v>
       </c>
       <c r="B4" t="s">
@@ -620,7 +628,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+      <c r="A5">
         <v>9288133</v>
       </c>
       <c r="B5" t="s">
@@ -634,7 +642,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+      <c r="A6">
         <v>9288134</v>
       </c>
       <c r="B6" t="s">
@@ -648,7 +656,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+      <c r="A7">
         <v>9288135</v>
       </c>
       <c r="B7" t="s">
@@ -662,7 +670,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
+      <c r="A8">
         <v>9288136</v>
       </c>
       <c r="B8" t="s">
@@ -676,7 +684,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+      <c r="A9">
         <v>9288137</v>
       </c>
       <c r="B9" t="s">
@@ -690,7 +698,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+      <c r="A10">
         <v>9288138</v>
       </c>
       <c r="B10" t="s">
@@ -704,7 +712,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
+      <c r="A11">
         <v>9288139</v>
       </c>
       <c r="B11" t="s">
@@ -718,7 +726,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
+      <c r="A12">
         <v>9288141</v>
       </c>
       <c r="B12" t="s">
@@ -732,7 +740,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
+      <c r="A13">
         <v>9288142</v>
       </c>
       <c r="B13" t="s">
@@ -746,7 +754,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
+      <c r="A14">
         <v>9288143</v>
       </c>
       <c r="B14" t="s">
@@ -760,7 +768,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
+      <c r="A15">
         <v>9288144</v>
       </c>
       <c r="B15" t="s">
@@ -774,7 +782,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4">
+      <c r="A16">
         <v>9288145</v>
       </c>
       <c r="B16" t="s">
@@ -788,7 +796,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4">
+      <c r="A17">
         <v>9288147</v>
       </c>
       <c r="B17" t="s">
@@ -802,7 +810,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
+      <c r="A18">
         <v>9288148</v>
       </c>
       <c r="B18" t="s">
@@ -816,7 +824,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4">
+      <c r="A19">
         <v>9288149</v>
       </c>
       <c r="B19" t="s">
@@ -830,7 +838,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
+      <c r="A20">
         <v>9288150</v>
       </c>
       <c r="B20" t="s">
@@ -844,7 +852,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
+      <c r="A21">
         <v>9288152</v>
       </c>
       <c r="B21" t="s">
@@ -858,7 +866,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
+      <c r="A22">
         <v>9288153</v>
       </c>
       <c r="B22" t="s">
@@ -872,7 +880,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
+      <c r="A23">
         <v>9288154</v>
       </c>
       <c r="B23" t="s">
@@ -886,7 +894,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
+      <c r="A24">
         <v>9288155</v>
       </c>
       <c r="B24" t="s">
@@ -900,7 +908,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
+      <c r="A25">
         <v>9288167</v>
       </c>
       <c r="B25" t="s">
@@ -914,7 +922,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
+      <c r="A26">
         <v>9288168</v>
       </c>
       <c r="B26" t="s">
@@ -928,7 +936,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
+      <c r="A27">
         <v>9288169</v>
       </c>
       <c r="B27" t="s">
@@ -943,7 +951,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
+      <c r="A28">
         <v>9288176</v>
       </c>
       <c r="B28" t="s">
@@ -957,7 +965,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="4">
+      <c r="A29">
         <v>9288177</v>
       </c>
       <c r="B29" t="s">
@@ -972,7 +980,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4">
+      <c r="A30">
         <v>9288178</v>
       </c>
       <c r="B30" t="s">
@@ -986,7 +994,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4">
+      <c r="A31">
         <v>9288179</v>
       </c>
       <c r="B31" t="s">
@@ -1000,7 +1008,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4">
+      <c r="A32">
         <v>9288180</v>
       </c>
       <c r="B32" t="s">
@@ -1014,7 +1022,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4">
+      <c r="A33">
         <v>9288181</v>
       </c>
       <c r="B33" t="s">
@@ -1028,7 +1036,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4">
+      <c r="A34">
         <v>9288182</v>
       </c>
       <c r="B34" t="s">
@@ -1042,7 +1050,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4">
+      <c r="A35">
         <v>9288183</v>
       </c>
       <c r="B35" t="s">
@@ -1056,7 +1064,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="4">
+      <c r="A36">
         <v>9288185</v>
       </c>
       <c r="B36" t="s">
@@ -1070,7 +1078,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="4">
+      <c r="A37">
         <v>9288186</v>
       </c>
       <c r="B37" t="s">
@@ -1084,7 +1092,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4">
+      <c r="A38">
         <v>9288187</v>
       </c>
       <c r="B38" t="s">
@@ -1098,7 +1106,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="4">
+      <c r="A39">
         <v>9288188</v>
       </c>
       <c r="B39" t="s">
@@ -1112,7 +1120,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="4">
+      <c r="A40">
         <v>9288189</v>
       </c>
       <c r="B40" t="s">
@@ -1126,7 +1134,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4">
+      <c r="A41">
         <v>9288190</v>
       </c>
       <c r="B41" t="s">
@@ -1140,7 +1148,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="4">
+      <c r="A42">
         <v>9288191</v>
       </c>
       <c r="B42" t="s">
@@ -1154,7 +1162,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="4">
+      <c r="A43">
         <v>9288192</v>
       </c>
       <c r="B43" t="s">
@@ -1168,7 +1176,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="4">
+      <c r="A44">
         <v>9288193</v>
       </c>
       <c r="B44" t="s">
@@ -1182,7 +1190,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="4">
+      <c r="A45">
         <v>9288194</v>
       </c>
       <c r="B45" t="s">
@@ -1196,7 +1204,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="4">
+      <c r="A46">
         <v>9288195</v>
       </c>
       <c r="B46" t="s">
@@ -1210,7 +1218,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="4">
+      <c r="A47">
         <v>9288196</v>
       </c>
       <c r="B47" t="s">
@@ -1224,7 +1232,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="4">
+      <c r="A48">
         <v>9288198</v>
       </c>
       <c r="B48" t="s">
@@ -1238,7 +1246,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="4">
+      <c r="A49">
         <v>9288209</v>
       </c>
       <c r="B49" t="s">
@@ -1252,7 +1260,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="4">
+      <c r="A50">
         <v>9288210</v>
       </c>
       <c r="B50" t="s">
@@ -1266,7 +1274,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="4">
+      <c r="A51">
         <v>9288211</v>
       </c>
       <c r="B51" t="s">
@@ -1280,7 +1288,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="4">
+      <c r="A52">
         <v>9288212</v>
       </c>
       <c r="B52" t="s">
@@ -1294,7 +1302,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="4">
+      <c r="A53">
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
@@ -1308,7 +1316,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="4">
+      <c r="A54">
         <v>9288214</v>
       </c>
       <c r="B54" t="s">
@@ -1322,7 +1330,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="4">
+      <c r="A55">
         <v>9321270</v>
       </c>
       <c r="B55" t="s">
@@ -1364,7 +1372,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState ref="A2:D57">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D57">
     <sortCondition ref="A1"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
altera formatação dos códigos
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D709A03-4578-4F6B-85D6-32EA7709D10B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19BC48AC-7097-4D8F-B26D-6944E7AD4E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="projetos" sheetId="9" r:id="rId1"/>
@@ -566,9 +566,8 @@
   <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="86.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="86.85546875" customWidth="1"/>
     <col min="4" max="4" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9.140625" style="1"/>
   </cols>

</xml_diff>

<commit_message>
Altera tipo para número
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90329DB9-EEFA-45C4-B1B2-7B63DBE2292D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BF8ECE-AF48-4B8F-A2A0-E235B045284F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -282,8 +282,8 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
preenche células em branco na coluna 1 para teste de conversão com formação correta
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25028"/>
-  <workbookPr hidePivotFieldList="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Silviana\Documents\1. CGE\tele-trabalho\GIT\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\Documents\teletrabalho\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05BF8ECE-AF48-4B8F-A2A0-E235B045284F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867"/>
   </bookViews>
   <sheets>
     <sheet name="projetos" sheetId="9" r:id="rId1"/>
@@ -232,7 +231,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
@@ -273,7 +272,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -286,6 +285,7 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -566,7 +566,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -592,7 +592,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4">
+      <c r="A2" s="6">
         <v>9288130</v>
       </c>
       <c r="B2" t="s">
@@ -606,7 +606,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
+      <c r="A3" s="6">
         <v>9288133</v>
       </c>
       <c r="B3" t="s">
@@ -620,7 +620,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="4">
+      <c r="A4" s="6">
         <v>9288134</v>
       </c>
       <c r="B4" t="s">
@@ -634,7 +634,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="4">
+      <c r="A5" s="6">
         <v>9288135</v>
       </c>
       <c r="B5" t="s">
@@ -648,7 +648,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="4">
+      <c r="A6" s="6">
         <v>9288136</v>
       </c>
       <c r="B6" t="s">
@@ -662,7 +662,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="4">
+      <c r="A7" s="6">
         <v>9288137</v>
       </c>
       <c r="B7" t="s">
@@ -676,7 +676,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4">
+      <c r="A8" s="6">
         <v>9288138</v>
       </c>
       <c r="B8" t="s">
@@ -690,7 +690,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="4">
+      <c r="A9" s="6">
         <v>9288139</v>
       </c>
       <c r="B9" t="s">
@@ -704,7 +704,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="4">
+      <c r="A10" s="6">
         <v>9288141</v>
       </c>
       <c r="B10" t="s">
@@ -718,7 +718,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="4">
+      <c r="A11" s="6">
         <v>9288142</v>
       </c>
       <c r="B11" t="s">
@@ -732,7 +732,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="4">
+      <c r="A12" s="6">
         <v>9288143</v>
       </c>
       <c r="B12" t="s">
@@ -746,7 +746,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="4">
+      <c r="A13" s="6">
         <v>9288144</v>
       </c>
       <c r="B13" t="s">
@@ -760,7 +760,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4">
+      <c r="A14" s="6">
         <v>9288145</v>
       </c>
       <c r="B14" t="s">
@@ -774,7 +774,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="4">
+      <c r="A15" s="6">
         <v>9288147</v>
       </c>
       <c r="B15" t="s">
@@ -788,7 +788,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="4">
+      <c r="A16" s="6">
         <v>9288148</v>
       </c>
       <c r="B16" t="s">
@@ -802,7 +802,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="4">
+      <c r="A17" s="6">
         <v>9288149</v>
       </c>
       <c r="B17" t="s">
@@ -816,7 +816,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="4">
+      <c r="A18" s="6">
         <v>9288150</v>
       </c>
       <c r="B18" t="s">
@@ -830,7 +830,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="4">
+      <c r="A19" s="6">
         <v>9288152</v>
       </c>
       <c r="B19" t="s">
@@ -844,7 +844,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
+      <c r="A20" s="6">
         <v>9288153</v>
       </c>
       <c r="B20" t="s">
@@ -858,7 +858,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
+      <c r="A21" s="6">
         <v>9288154</v>
       </c>
       <c r="B21" t="s">
@@ -872,7 +872,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
+      <c r="A22" s="6">
         <v>9288155</v>
       </c>
       <c r="B22" t="s">
@@ -886,7 +886,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="4">
+      <c r="A23" s="6">
         <v>9288167</v>
       </c>
       <c r="B23" t="s">
@@ -900,7 +900,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="4">
+      <c r="A24" s="6">
         <v>9288168</v>
       </c>
       <c r="B24" t="s">
@@ -914,7 +914,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="4">
+      <c r="A25" s="6">
         <v>9288169</v>
       </c>
       <c r="B25" t="s">
@@ -928,7 +928,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="4">
+      <c r="A26" s="6">
         <v>9288176</v>
       </c>
       <c r="B26" t="s">
@@ -943,7 +943,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="4">
+      <c r="A27" s="6">
         <v>9288177</v>
       </c>
       <c r="B27" t="s">
@@ -957,7 +957,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="4">
+      <c r="A28" s="6">
         <v>9288177</v>
       </c>
       <c r="B28" t="s">
@@ -972,7 +972,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="4">
+      <c r="A29" s="6">
         <v>9288178</v>
       </c>
       <c r="B29" t="s">
@@ -986,7 +986,7 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="4">
+      <c r="A30" s="6">
         <v>9288179</v>
       </c>
       <c r="B30" t="s">
@@ -1000,7 +1000,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4">
+      <c r="A31" s="6">
         <v>9288180</v>
       </c>
       <c r="B31" t="s">
@@ -1014,7 +1014,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4">
+      <c r="A32" s="6">
         <v>9288181</v>
       </c>
       <c r="B32" t="s">
@@ -1028,7 +1028,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="4">
+      <c r="A33" s="6">
         <v>9288182</v>
       </c>
       <c r="B33" t="s">
@@ -1042,7 +1042,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="4">
+      <c r="A34" s="6">
         <v>9288182</v>
       </c>
       <c r="B34" t="s">
@@ -1056,7 +1056,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="4">
+      <c r="A35" s="6">
         <v>9288183</v>
       </c>
       <c r="B35" t="s">
@@ -1070,7 +1070,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="4">
+      <c r="A36" s="6">
         <v>9288185</v>
       </c>
       <c r="B36" t="s">
@@ -1084,7 +1084,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="4">
+      <c r="A37" s="6">
         <v>9288186</v>
       </c>
       <c r="B37" t="s">
@@ -1098,7 +1098,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4">
+      <c r="A38" s="6">
         <v>9288187</v>
       </c>
       <c r="B38" t="s">
@@ -1112,7 +1112,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="4">
+      <c r="A39" s="6">
         <v>9288188</v>
       </c>
       <c r="B39" t="s">
@@ -1126,7 +1126,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="4">
+      <c r="A40" s="6">
         <v>9288189</v>
       </c>
       <c r="B40" t="s">
@@ -1140,7 +1140,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4">
+      <c r="A41" s="6">
         <v>9288190</v>
       </c>
       <c r="B41" t="s">
@@ -1154,7 +1154,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="4">
+      <c r="A42" s="6">
         <v>9288191</v>
       </c>
       <c r="B42" t="s">
@@ -1168,7 +1168,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="4">
+      <c r="A43" s="6">
         <v>9288192</v>
       </c>
       <c r="B43" t="s">
@@ -1182,7 +1182,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="4">
+      <c r="A44" s="6">
         <v>9288193</v>
       </c>
       <c r="B44" t="s">
@@ -1196,7 +1196,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="4">
+      <c r="A45" s="6">
         <v>9288194</v>
       </c>
       <c r="B45" t="s">
@@ -1210,7 +1210,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="4">
+      <c r="A46" s="6">
         <v>9288195</v>
       </c>
       <c r="B46" t="s">
@@ -1224,7 +1224,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="4">
+      <c r="A47" s="6">
         <v>9288196</v>
       </c>
       <c r="B47" t="s">
@@ -1238,7 +1238,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="4">
+      <c r="A48" s="6">
         <v>9288198</v>
       </c>
       <c r="B48" t="s">
@@ -1252,7 +1252,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="4">
+      <c r="A49" s="6">
         <v>9288209</v>
       </c>
       <c r="B49" t="s">
@@ -1266,7 +1266,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="4">
+      <c r="A50" s="6">
         <v>9288210</v>
       </c>
       <c r="B50" t="s">
@@ -1280,7 +1280,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="4">
+      <c r="A51" s="6">
         <v>9288211</v>
       </c>
       <c r="B51" t="s">
@@ -1294,7 +1294,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="4">
+      <c r="A52" s="6">
         <v>9288212</v>
       </c>
       <c r="B52" t="s">
@@ -1308,7 +1308,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="4">
+      <c r="A53" s="6">
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
@@ -1322,7 +1322,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="4">
+      <c r="A54" s="6">
         <v>9288214</v>
       </c>
       <c r="B54" t="s">
@@ -1336,7 +1336,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="4">
+      <c r="A55" s="6">
         <v>9321270</v>
       </c>
       <c r="B55" t="s">
@@ -1350,7 +1350,9 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
+      <c r="A56" s="6">
+        <v>9288214</v>
+      </c>
       <c r="B56" t="s">
         <v>5</v>
       </c>
@@ -1362,7 +1364,9 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="4"/>
+      <c r="A57" s="6">
+        <v>9321270</v>
+      </c>
       <c r="B57" t="s">
         <v>29</v>
       </c>
@@ -1374,7 +1378,7 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D57">
+  <sortState ref="A2:D57">
     <sortCondition ref="A2:A57"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Add file with validation error
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -42,6 +42,9 @@
     <t>Elaboração de Plano Metropolitano de Segurança Hídrica para a Região Metropolitana de Belo Horizonte.</t>
   </si>
   <si>
+    <t>Intervenções e Obras a serem realizadas, sob a responsabilidade e de propriedade do Estado de Minas Gerais, com o objetivo de aumentar a resiliência das Bacias do Paraopeba e Rio das Velhas, de modo a garantir o abastecimento da Região Metropolitana de Belo Horizonte - RMBH.</t>
+  </si>
+  <si>
     <t>III</t>
   </si>
   <si>
@@ -223,9 +226,6 @@
   </si>
   <si>
     <t>valor_projeto</t>
-  </si>
-  <si>
-    <t>Intervenções e Obras a serem realizadas, sob a responsabilidade e de propriedade do Estado de Minas Gerais, com o objetivo de aumentar a resiliência das Bacias do Paraopeba e Rio das Velhas, de modo a garantir o abastecimento da Região Metropolitana de Belo Horizonte - RMBH</t>
   </si>
 </sst>
 </file>
@@ -579,16 +579,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -596,10 +596,10 @@
         <v>9288130</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
       </c>
       <c r="D2" s="3">
         <v>450000000</v>
@@ -610,10 +610,10 @@
         <v>9288133</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="3">
         <v>700000000</v>
@@ -624,10 +624,10 @@
         <v>9288134</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3">
         <v>98860000</v>
@@ -638,10 +638,10 @@
         <v>9288135</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3">
         <v>1345000</v>
@@ -652,10 +652,10 @@
         <v>9288136</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3">
         <v>111480000</v>
@@ -666,10 +666,10 @@
         <v>9288137</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D7" s="3">
         <v>100000000</v>
@@ -680,10 +680,10 @@
         <v>9288138</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="3">
         <v>39614000</v>
@@ -694,10 +694,10 @@
         <v>9288139</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="3">
         <v>3200000</v>
@@ -708,10 +708,10 @@
         <v>9288141</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D10" s="3">
         <v>500000</v>
@@ -722,10 +722,10 @@
         <v>9288142</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="3">
         <v>29712000</v>
@@ -736,10 +736,10 @@
         <v>9288143</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3">
         <v>728000</v>
@@ -750,10 +750,10 @@
         <v>9288144</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D13" s="3">
         <v>49000000</v>
@@ -764,10 +764,10 @@
         <v>9288145</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D14" s="3">
         <v>45345000</v>
@@ -778,10 +778,10 @@
         <v>9288147</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D15" s="3">
         <v>14817323</v>
@@ -792,10 +792,10 @@
         <v>9288148</v>
       </c>
       <c r="B16" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D16" s="3">
         <v>3000000</v>
@@ -806,10 +806,10 @@
         <v>9288149</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D17" s="3">
         <v>5000000</v>
@@ -820,10 +820,10 @@
         <v>9288150</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D18" s="3">
         <v>10671300</v>
@@ -834,10 +834,10 @@
         <v>9288152</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D19" s="3">
         <v>15130000</v>
@@ -848,10 +848,10 @@
         <v>9288153</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D20" s="3">
         <v>3000000</v>
@@ -862,10 +862,10 @@
         <v>9288154</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D21" s="3">
         <v>650000</v>
@@ -876,10 +876,10 @@
         <v>9288155</v>
       </c>
       <c r="B22" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D22" s="3">
         <v>5100000</v>
@@ -890,10 +890,10 @@
         <v>9288167</v>
       </c>
       <c r="B23" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" s="3">
         <v>3773400</v>
@@ -904,10 +904,10 @@
         <v>9288168</v>
       </c>
       <c r="B24" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D24" s="3">
         <v>130000000</v>
@@ -918,10 +918,10 @@
         <v>9288169</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" s="3">
         <v>43368482</v>
@@ -932,10 +932,10 @@
         <v>9288176</v>
       </c>
       <c r="B26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C26" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D26" s="3">
         <f>8700000+14431467.96</f>
@@ -947,10 +947,10 @@
         <v>9288177</v>
       </c>
       <c r="B27" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27" s="3">
         <v>100370000</v>
@@ -961,10 +961,10 @@
         <v>9288177</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D28" s="3">
         <f>1048250000+59300000</f>
@@ -976,10 +976,10 @@
         <v>9288178</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C29" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D29" s="3">
         <v>253000000</v>
@@ -990,10 +990,10 @@
         <v>9288179</v>
       </c>
       <c r="B30" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D30" s="3">
         <v>45000000</v>
@@ -1004,10 +1004,10 @@
         <v>9288180</v>
       </c>
       <c r="B31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C31" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D31" s="3">
         <v>3072030000</v>
@@ -1018,10 +1018,10 @@
         <v>9288181</v>
       </c>
       <c r="B32" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C32" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D32" s="3">
         <v>75352000</v>
@@ -1032,10 +1032,10 @@
         <v>9288182</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C33" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D33" s="3">
         <v>300000000</v>
@@ -1046,10 +1046,10 @@
         <v>9288182</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D34" s="3">
         <v>7000000</v>
@@ -1060,10 +1060,10 @@
         <v>9288183</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C35" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D35" s="3">
         <v>8000000</v>
@@ -1077,7 +1077,7 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D36" s="3">
         <v>2000000</v>
@@ -1088,10 +1088,10 @@
         <v>9288186</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C37" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D37" s="3">
         <v>3000000</v>
@@ -1102,10 +1102,10 @@
         <v>9288187</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C38" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D38" s="3">
         <v>36000000</v>
@@ -1116,10 +1116,10 @@
         <v>9288188</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C39" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D39" s="3">
         <v>8647600</v>
@@ -1130,10 +1130,10 @@
         <v>9288189</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D40" s="3">
         <v>300000</v>
@@ -1144,10 +1144,10 @@
         <v>9288190</v>
       </c>
       <c r="B41" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C41" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D41" s="3">
         <v>100000000</v>
@@ -1158,10 +1158,10 @@
         <v>9288191</v>
       </c>
       <c r="B42" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D42" s="3">
         <v>210000000</v>
@@ -1172,10 +1172,10 @@
         <v>9288192</v>
       </c>
       <c r="B43" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C43" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D43" s="3">
         <v>100000000</v>
@@ -1186,10 +1186,10 @@
         <v>9288193</v>
       </c>
       <c r="B44" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C44" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D44" s="3">
         <v>3900000</v>
@@ -1200,10 +1200,10 @@
         <v>9288194</v>
       </c>
       <c r="B45" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C45" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D45" s="3">
         <v>3600000</v>
@@ -1214,10 +1214,10 @@
         <v>9288195</v>
       </c>
       <c r="B46" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D46" s="3">
         <v>749679</v>
@@ -1228,10 +1228,10 @@
         <v>9288196</v>
       </c>
       <c r="B47" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C47" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D47" s="3">
         <v>42412000</v>
@@ -1242,10 +1242,10 @@
         <v>9288198</v>
       </c>
       <c r="B48" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C48" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D48" s="3">
         <v>985935044</v>
@@ -1256,10 +1256,10 @@
         <v>9288209</v>
       </c>
       <c r="B49" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C49" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D49" s="3">
         <v>1200000</v>
@@ -1270,10 +1270,10 @@
         <v>9288210</v>
       </c>
       <c r="B50" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C50" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D50" s="3">
         <v>2500000</v>
@@ -1284,10 +1284,10 @@
         <v>9288211</v>
       </c>
       <c r="B51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C51" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D51" s="3">
         <v>3200000</v>
@@ -1298,7 +1298,7 @@
         <v>9288212</v>
       </c>
       <c r="B52" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="C52" t="s">
         <v>0</v>
@@ -1312,10 +1312,10 @@
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D53" s="3">
         <v>23000005</v>
@@ -1326,10 +1326,10 @@
         <v>9288214</v>
       </c>
       <c r="B54" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C54" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D54" s="3">
         <v>199489167.000002</v>
@@ -1340,10 +1340,10 @@
         <v>9321270</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C55" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D55" s="3">
         <v>800000</v>
@@ -1354,10 +1354,10 @@
         <v>9288214</v>
       </c>
       <c r="B56" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D56" s="3">
         <v>427970000</v>
@@ -1368,10 +1368,10 @@
         <v>9321270</v>
       </c>
       <c r="B57" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C57" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D57" s="3">
         <v>14000000</v>

</xml_diff>

<commit_message>
Projetos Acordo Judicial de Reparação da Vale
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="64">
   <si>
     <t>II.3</t>
   </si>
@@ -212,6 +212,9 @@
   </si>
   <si>
     <t>Intervenções e Obras a serem realizadas, sob a responsabilidade e de propriedade do Estado de Minas Gerais, com o objetivo de aumentar a resiliência das Bacias do Paraopeba e Rio das Velhas, de modo a garantir o abastecimento da Região Metropolitana de Belo Horizonte - RMBH</t>
+  </si>
+  <si>
+    <t>Complementação dos recursos federais para o Metrô da RMBH</t>
   </si>
 </sst>
 </file>
@@ -258,7 +261,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -273,6 +276,7 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,7 +550,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -554,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1350,6 +1354,20 @@
       </c>
       <c r="D56" s="3">
         <v>14000000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="A57" s="1">
+        <v>9999999</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D57" s="2">
+        <v>427970000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Renomeia conjunto de dados
Fix #7
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -239,7 +239,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,6 +248,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -276,7 +284,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -292,6 +300,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="1"/>
@@ -1372,6 +1383,9 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>9999999</v>
+      </c>
       <c r="B57" s="6" t="s">
         <v>63</v>
       </c>
@@ -1381,6 +1395,9 @@
       <c r="D57" s="2">
         <v>427970000</v>
       </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualização conforme Deliberação 7 e 8 de 2022
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -1,13 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\tele-trabalho\transparencia-mg\acordo-judicial-reparacao-vale\upload\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+  <workbookPr hidePivotFieldList="1"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="867"/>
   </bookViews>
@@ -16,9 +11,9 @@
     <sheet name="Plan1" sheetId="10" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">projetos!$A$1:$D$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">projetos!$A$1:$L$60</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="144525"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +25,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="67">
   <si>
     <t>II.3</t>
   </si>
@@ -230,16 +224,25 @@
   </si>
   <si>
     <t>Complementação dos recursos federais para o Metrô da RMBH</t>
+  </si>
+  <si>
+    <t>Ampliação da capacidade de cobertura da malha aérea da Polícia Militar de Minas Gerais</t>
+  </si>
+  <si>
+    <t>Melhoria da infraestrutura dos municípios - Mobilidade regional na Bacia do Paraopeba</t>
+  </si>
+  <si>
+    <t>Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG / conclusão de corredor logístico estruturante, conforme critérios técnicos da Seinfra - Mobilidade regional na Bacia do Paraopeba</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -254,21 +257,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -284,7 +285,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -300,8 +301,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -364,7 +376,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -399,7 +411,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -576,7 +588,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -584,11 +596,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="29" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="62.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" style="1"/>
     <col min="4" max="4" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="11" width="9.140625" style="1"/>
@@ -597,7 +609,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="7" t="s">
         <v>57</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -611,36 +623,36 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="8">
         <v>9288130</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3">
-        <v>450000000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>9288130</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="3">
         <f>1048250000+59300000</f>
         <v>1107550000</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>9288130</v>
+      </c>
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="3">
+        <v>450000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
         <v>9288132</v>
       </c>
       <c r="B4" t="s">
@@ -654,7 +666,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="8">
         <v>9288133</v>
       </c>
       <c r="B5" t="s">
@@ -668,7 +680,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="8">
         <v>9288134</v>
       </c>
       <c r="B6" t="s">
@@ -682,7 +694,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="8">
         <v>9288135</v>
       </c>
       <c r="B7" t="s">
@@ -696,7 +708,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="8">
         <v>9288136</v>
       </c>
       <c r="B8" t="s">
@@ -710,7 +722,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="8">
         <v>9288137</v>
       </c>
       <c r="B9" t="s">
@@ -724,7 +736,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="8">
         <v>9288138</v>
       </c>
       <c r="B10" t="s">
@@ -738,7 +750,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="8">
         <v>9288139</v>
       </c>
       <c r="B11" t="s">
@@ -752,7 +764,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="8">
         <v>9288141</v>
       </c>
       <c r="B12" t="s">
@@ -766,7 +778,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="A13" s="8">
         <v>9288142</v>
       </c>
       <c r="B13" t="s">
@@ -780,7 +792,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="A14" s="8">
         <v>9288143</v>
       </c>
       <c r="B14" t="s">
@@ -794,7 +806,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="A15" s="8">
         <v>9288144</v>
       </c>
       <c r="B15" t="s">
@@ -808,7 +820,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="A16" s="8">
         <v>9288145</v>
       </c>
       <c r="B16" t="s">
@@ -822,7 +834,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="A17" s="8">
         <v>9288147</v>
       </c>
       <c r="B17" t="s">
@@ -836,7 +848,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="A18" s="8">
         <v>9288148</v>
       </c>
       <c r="B18" t="s">
@@ -850,7 +862,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="A19" s="8">
         <v>9288149</v>
       </c>
       <c r="B19" t="s">
@@ -864,7 +876,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20">
+      <c r="A20" s="8">
         <v>9288150</v>
       </c>
       <c r="B20" t="s">
@@ -878,7 +890,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21">
+      <c r="A21" s="8">
         <v>9288152</v>
       </c>
       <c r="B21" t="s">
@@ -892,7 +904,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="A22" s="8">
         <v>9288153</v>
       </c>
       <c r="B22" t="s">
@@ -906,7 +918,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="A23" s="8">
         <v>9288154</v>
       </c>
       <c r="B23" t="s">
@@ -920,7 +932,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24">
+      <c r="A24" s="8">
         <v>9288155</v>
       </c>
       <c r="B24" t="s">
@@ -934,7 +946,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25">
+      <c r="A25" s="8">
         <v>9288167</v>
       </c>
       <c r="B25" t="s">
@@ -948,7 +960,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26">
+      <c r="A26" s="8">
         <v>9288168</v>
       </c>
       <c r="B26" t="s">
@@ -962,7 +974,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27">
+      <c r="A27" s="8">
         <v>9288169</v>
       </c>
       <c r="B27" t="s">
@@ -976,7 +988,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="A28" s="8">
         <v>9288176</v>
       </c>
       <c r="B28" t="s">
@@ -991,7 +1003,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29">
+      <c r="A29" s="8">
         <v>9288177</v>
       </c>
       <c r="B29" t="s">
@@ -1000,12 +1012,12 @@
       <c r="C29" t="s">
         <v>7</v>
       </c>
-      <c r="D29" s="3">
-        <v>100370000</v>
+      <c r="D29" s="11">
+        <v>88370000</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30">
+      <c r="A30" s="8">
         <v>9288178</v>
       </c>
       <c r="B30" t="s">
@@ -1019,7 +1031,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31">
+      <c r="A31" s="8">
         <v>9288179</v>
       </c>
       <c r="B31" t="s">
@@ -1033,7 +1045,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32">
+      <c r="A32" s="8">
         <v>9288180</v>
       </c>
       <c r="B32" t="s">
@@ -1047,7 +1059,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33">
+      <c r="A33" s="8">
         <v>9288181</v>
       </c>
       <c r="B33" t="s">
@@ -1061,7 +1073,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34">
+      <c r="A34" s="8">
         <v>9288182</v>
       </c>
       <c r="B34" t="s">
@@ -1075,7 +1087,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35">
+      <c r="A35" s="8">
         <v>9288183</v>
       </c>
       <c r="B35" t="s">
@@ -1089,7 +1101,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
+      <c r="A36" s="8">
         <v>9288185</v>
       </c>
       <c r="B36" t="s">
@@ -1103,7 +1115,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37">
+      <c r="A37" s="8">
         <v>9288186</v>
       </c>
       <c r="B37" t="s">
@@ -1117,7 +1129,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38">
+      <c r="A38" s="8">
         <v>9288187</v>
       </c>
       <c r="B38" t="s">
@@ -1131,7 +1143,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39">
+      <c r="A39" s="8">
         <v>9288188</v>
       </c>
       <c r="B39" t="s">
@@ -1145,7 +1157,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40">
+      <c r="A40" s="8">
         <v>9288189</v>
       </c>
       <c r="B40" t="s">
@@ -1159,7 +1171,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41">
+      <c r="A41" s="8">
         <v>9288190</v>
       </c>
       <c r="B41" t="s">
@@ -1173,7 +1185,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42">
+      <c r="A42" s="8">
         <v>9288191</v>
       </c>
       <c r="B42" t="s">
@@ -1187,7 +1199,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43">
+      <c r="A43" s="8">
         <v>9288192</v>
       </c>
       <c r="B43" t="s">
@@ -1201,7 +1213,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44">
+      <c r="A44" s="8">
         <v>9288193</v>
       </c>
       <c r="B44" t="s">
@@ -1215,7 +1227,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45">
+      <c r="A45" s="8">
         <v>9288194</v>
       </c>
       <c r="B45" t="s">
@@ -1229,7 +1241,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46">
+      <c r="A46" s="8">
         <v>9288195</v>
       </c>
       <c r="B46" t="s">
@@ -1243,7 +1255,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47">
+      <c r="A47" s="8">
         <v>9288196</v>
       </c>
       <c r="B47" t="s">
@@ -1257,7 +1269,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48">
+      <c r="A48" s="8">
         <v>9288198</v>
       </c>
       <c r="B48" t="s">
@@ -1271,7 +1283,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49">
+      <c r="A49" s="8">
         <v>9288209</v>
       </c>
       <c r="B49" t="s">
@@ -1285,7 +1297,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50">
+      <c r="A50" s="8">
         <v>9288210</v>
       </c>
       <c r="B50" t="s">
@@ -1299,7 +1311,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51">
+      <c r="A51" s="8">
         <v>9288211</v>
       </c>
       <c r="B51" t="s">
@@ -1313,7 +1325,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52">
+      <c r="A52" s="8">
         <v>9288212</v>
       </c>
       <c r="B52" t="s">
@@ -1327,7 +1339,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53">
+      <c r="A53" s="8">
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
@@ -1341,7 +1353,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54">
+      <c r="A54" s="8">
         <v>9288214</v>
       </c>
       <c r="B54" t="s">
@@ -1355,7 +1367,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55">
+      <c r="A55" s="8">
         <v>9321270</v>
       </c>
       <c r="B55" t="s">
@@ -1369,7 +1381,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56">
+      <c r="A56" s="8">
         <v>9334530</v>
       </c>
       <c r="B56" t="s">
@@ -1383,8 +1395,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
-        <v>9999999</v>
+      <c r="A57" s="12">
+        <v>9337957</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>63</v>
@@ -1397,9 +1409,51 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
+      <c r="A58" s="8">
+        <v>9341846</v>
+      </c>
+      <c r="B58" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" t="s">
+        <v>7</v>
+      </c>
+      <c r="D58" s="3">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59" s="8">
+        <v>9999999</v>
+      </c>
+      <c r="B59" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59" s="3">
+        <v>56352383.469999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60" s="8">
+        <v>9999999</v>
+      </c>
+      <c r="B60" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2</v>
+      </c>
+      <c r="D60" s="3">
+        <v>47997269.119999997</v>
+      </c>
     </row>
   </sheetData>
+  <sortState ref="A2:D61">
+    <sortCondition ref="A1:A61"/>
+  </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza arquivo conforme a Deliberação 8.
Adiciona o número do instrumento do projeto "Mobilidade regional na Bacia do Paraopeba" previsto na Deliberação 8 do Conselho Superior Pró Brumadinho. 
"
</commit_message>
<xml_diff>
--- a/upload/projetos_acordo_judicial_reparacao_vale.xlsx
+++ b/upload/projetos_acordo_judicial_reparacao_vale.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="67">
   <si>
     <t>II.3</t>
   </si>
@@ -229,10 +229,10 @@
     <t>Ampliação da capacidade de cobertura da malha aérea da Polícia Militar de Minas Gerais</t>
   </si>
   <si>
-    <t>Melhoria da infraestrutura dos municípios - Mobilidade regional na Bacia do Paraopeba</t>
-  </si>
-  <si>
-    <t>Recuperação de rodovias pavimentadas em pior estado, conforme avaliação técnica do DER-MG / conclusão de corredor logístico estruturante, conforme critérios técnicos da Seinfra - Mobilidade regional na Bacia do Paraopeba</t>
+    <t>Mobilidade regional na Bacia do Paraopeba</t>
+  </si>
+  <si>
+    <t>III e IV</t>
   </si>
 </sst>
 </file>
@@ -285,7 +285,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -300,7 +300,6 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -310,11 +309,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,7 +583,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -596,10 +591,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="14.28515625" style="8" customWidth="1"/>
     <col min="2" max="2" width="62.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.140625" style="1"/>
     <col min="4" max="4" width="17.7109375" style="2" bestFit="1" customWidth="1"/>
@@ -609,7 +604,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B1" s="4" t="s">
@@ -623,7 +618,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2" s="7">
         <v>9288130</v>
       </c>
       <c r="B2" t="s">
@@ -638,7 +633,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="7">
         <v>9288130</v>
       </c>
       <c r="B3" t="s">
@@ -652,7 +647,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+      <c r="A4" s="7">
         <v>9288132</v>
       </c>
       <c r="B4" t="s">
@@ -666,7 +661,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+      <c r="A5" s="7">
         <v>9288133</v>
       </c>
       <c r="B5" t="s">
@@ -680,7 +675,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+      <c r="A6" s="7">
         <v>9288134</v>
       </c>
       <c r="B6" t="s">
@@ -694,7 +689,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>9288135</v>
       </c>
       <c r="B7" t="s">
@@ -708,7 +703,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+      <c r="A8" s="7">
         <v>9288136</v>
       </c>
       <c r="B8" t="s">
@@ -722,7 +717,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="8">
+      <c r="A9" s="7">
         <v>9288137</v>
       </c>
       <c r="B9" t="s">
@@ -736,7 +731,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="8">
+      <c r="A10" s="7">
         <v>9288138</v>
       </c>
       <c r="B10" t="s">
@@ -750,7 +745,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8">
+      <c r="A11" s="7">
         <v>9288139</v>
       </c>
       <c r="B11" t="s">
@@ -764,7 +759,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="8">
+      <c r="A12" s="7">
         <v>9288141</v>
       </c>
       <c r="B12" t="s">
@@ -778,7 +773,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>9288142</v>
       </c>
       <c r="B13" t="s">
@@ -792,7 +787,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8">
+      <c r="A14" s="7">
         <v>9288143</v>
       </c>
       <c r="B14" t="s">
@@ -806,7 +801,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8">
+      <c r="A15" s="7">
         <v>9288144</v>
       </c>
       <c r="B15" t="s">
@@ -820,7 +815,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8">
+      <c r="A16" s="7">
         <v>9288145</v>
       </c>
       <c r="B16" t="s">
@@ -834,7 +829,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8">
+      <c r="A17" s="7">
         <v>9288147</v>
       </c>
       <c r="B17" t="s">
@@ -848,7 +843,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8">
+      <c r="A18" s="7">
         <v>9288148</v>
       </c>
       <c r="B18" t="s">
@@ -862,7 +857,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="8">
+      <c r="A19" s="7">
         <v>9288149</v>
       </c>
       <c r="B19" t="s">
@@ -876,7 +871,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="8">
+      <c r="A20" s="7">
         <v>9288150</v>
       </c>
       <c r="B20" t="s">
@@ -890,7 +885,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="8">
+      <c r="A21" s="7">
         <v>9288152</v>
       </c>
       <c r="B21" t="s">
@@ -904,7 +899,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="A22" s="7">
         <v>9288153</v>
       </c>
       <c r="B22" t="s">
@@ -918,7 +913,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
+      <c r="A23" s="7">
         <v>9288154</v>
       </c>
       <c r="B23" t="s">
@@ -932,7 +927,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
+      <c r="A24" s="7">
         <v>9288155</v>
       </c>
       <c r="B24" t="s">
@@ -946,7 +941,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
+      <c r="A25" s="7">
         <v>9288167</v>
       </c>
       <c r="B25" t="s">
@@ -960,7 +955,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="8">
+      <c r="A26" s="7">
         <v>9288168</v>
       </c>
       <c r="B26" t="s">
@@ -974,7 +969,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="8">
+      <c r="A27" s="7">
         <v>9288169</v>
       </c>
       <c r="B27" t="s">
@@ -988,7 +983,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="8">
+      <c r="A28" s="7">
         <v>9288176</v>
       </c>
       <c r="B28" t="s">
@@ -1003,7 +998,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="8">
+      <c r="A29" s="7">
         <v>9288177</v>
       </c>
       <c r="B29" t="s">
@@ -1012,12 +1007,12 @@
       <c r="C29" t="s">
         <v>7</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="9">
         <v>88370000</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="8">
+      <c r="A30" s="7">
         <v>9288178</v>
       </c>
       <c r="B30" t="s">
@@ -1031,7 +1026,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="8">
+      <c r="A31" s="7">
         <v>9288179</v>
       </c>
       <c r="B31" t="s">
@@ -1045,7 +1040,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="8">
+      <c r="A32" s="7">
         <v>9288180</v>
       </c>
       <c r="B32" t="s">
@@ -1059,7 +1054,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="8">
+      <c r="A33" s="7">
         <v>9288181</v>
       </c>
       <c r="B33" t="s">
@@ -1073,7 +1068,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="8">
+      <c r="A34" s="7">
         <v>9288182</v>
       </c>
       <c r="B34" t="s">
@@ -1087,7 +1082,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="8">
+      <c r="A35" s="7">
         <v>9288183</v>
       </c>
       <c r="B35" t="s">
@@ -1101,7 +1096,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="8">
+      <c r="A36" s="7">
         <v>9288185</v>
       </c>
       <c r="B36" t="s">
@@ -1115,7 +1110,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="8">
+      <c r="A37" s="7">
         <v>9288186</v>
       </c>
       <c r="B37" t="s">
@@ -1129,7 +1124,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="8">
+      <c r="A38" s="7">
         <v>9288187</v>
       </c>
       <c r="B38" t="s">
@@ -1143,7 +1138,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="8">
+      <c r="A39" s="7">
         <v>9288188</v>
       </c>
       <c r="B39" t="s">
@@ -1157,7 +1152,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="8">
+      <c r="A40" s="7">
         <v>9288189</v>
       </c>
       <c r="B40" t="s">
@@ -1171,7 +1166,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="8">
+      <c r="A41" s="7">
         <v>9288190</v>
       </c>
       <c r="B41" t="s">
@@ -1185,7 +1180,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="8">
+      <c r="A42" s="7">
         <v>9288191</v>
       </c>
       <c r="B42" t="s">
@@ -1199,7 +1194,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="8">
+      <c r="A43" s="7">
         <v>9288192</v>
       </c>
       <c r="B43" t="s">
@@ -1213,7 +1208,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="8">
+      <c r="A44" s="7">
         <v>9288193</v>
       </c>
       <c r="B44" t="s">
@@ -1227,7 +1222,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="8">
+      <c r="A45" s="7">
         <v>9288194</v>
       </c>
       <c r="B45" t="s">
@@ -1241,7 +1236,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="8">
+      <c r="A46" s="7">
         <v>9288195</v>
       </c>
       <c r="B46" t="s">
@@ -1255,7 +1250,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="8">
+      <c r="A47" s="7">
         <v>9288196</v>
       </c>
       <c r="B47" t="s">
@@ -1269,7 +1264,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="8">
+      <c r="A48" s="7">
         <v>9288198</v>
       </c>
       <c r="B48" t="s">
@@ -1283,7 +1278,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="8">
+      <c r="A49" s="7">
         <v>9288209</v>
       </c>
       <c r="B49" t="s">
@@ -1297,7 +1292,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="8">
+      <c r="A50" s="7">
         <v>9288210</v>
       </c>
       <c r="B50" t="s">
@@ -1311,7 +1306,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="8">
+      <c r="A51" s="7">
         <v>9288211</v>
       </c>
       <c r="B51" t="s">
@@ -1325,7 +1320,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="8">
+      <c r="A52" s="7">
         <v>9288212</v>
       </c>
       <c r="B52" t="s">
@@ -1339,7 +1334,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="8">
+      <c r="A53" s="7">
         <v>9288213</v>
       </c>
       <c r="B53" t="s">
@@ -1353,7 +1348,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="8">
+      <c r="A54" s="7">
         <v>9288214</v>
       </c>
       <c r="B54" t="s">
@@ -1367,7 +1362,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="8">
+      <c r="A55" s="7">
         <v>9321270</v>
       </c>
       <c r="B55" t="s">
@@ -1381,7 +1376,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="8">
+      <c r="A56" s="7">
         <v>9334530</v>
       </c>
       <c r="B56" t="s">
@@ -1395,24 +1390,24 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="12">
+      <c r="A57" s="7">
         <v>9337957</v>
       </c>
-      <c r="B57" s="6" t="s">
+      <c r="B57" t="s">
         <v>63</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" t="s">
         <v>2</v>
       </c>
-      <c r="D57" s="2">
+      <c r="D57" s="3">
         <v>427970000</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="8">
+      <c r="A58" s="7">
         <v>9341846</v>
       </c>
-      <c r="B58" s="10" t="s">
+      <c r="B58" t="s">
         <v>64</v>
       </c>
       <c r="C58" t="s">
@@ -1423,32 +1418,36 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="8">
-        <v>9999999</v>
-      </c>
-      <c r="B59" s="10" t="s">
+      <c r="A59" s="7">
+        <v>9342884</v>
+      </c>
+      <c r="B59" t="s">
         <v>65</v>
       </c>
       <c r="C59" t="s">
-        <v>7</v>
+        <v>66</v>
       </c>
       <c r="D59" s="3">
-        <v>56352383.469999999</v>
+        <v>104349652.59</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="8">
-        <v>9999999</v>
-      </c>
-      <c r="B60" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="C60" t="s">
-        <v>2</v>
-      </c>
-      <c r="D60" s="3">
-        <v>47997269.119999997</v>
-      </c>
+      <c r="A60" s="7"/>
+      <c r="B60"/>
+      <c r="C60"/>
+      <c r="D60" s="3"/>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61" s="7"/>
+      <c r="B61"/>
+      <c r="C61"/>
+      <c r="D61" s="3"/>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62"/>
+      <c r="C62"/>
+      <c r="D62" s="3"/>
     </row>
   </sheetData>
   <sortState ref="A2:D61">

</xml_diff>